<commit_message>
docs(roadmap): record the reskin sweep and the defects it surfaced
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dobby_100_Day_Roadmap.xlsx
+++ b/Dobby_100_Day_Roadmap.xlsx
@@ -14201,7 +14201,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -14639,7 +14639,7 @@
       </c>
       <c r="D12" s="154" t="inlineStr">
         <is>
-          <t>Delivered: warm-paper/navy token pair, serif display face, Daily Alignment hero on Today (date, greeting, ruled outcome, numbered plan), left-rule nav, React Flow chrome themed.</t>
+          <t>Delivered across all 29 pages: warm-paper/navy token pair, serif display face, Daily Alignment hero on Today, route-derived eyebrows, action on the title row, React Flow chrome themed. Sweep also fixed four defects — see row 43.</t>
         </is>
       </c>
       <c r="E12" s="154" t="inlineStr">
@@ -15858,6 +15858,46 @@
         </is>
       </c>
       <c r="H42" s="142" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="126" t="n">
+        <v>43</v>
+      </c>
+      <c r="B43" s="142" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="C43" s="142" t="inlineStr">
+        <is>
+          <t>Timestamps, charts and graph layout fixed during the page-by-page sweep</t>
+        </is>
+      </c>
+      <c r="D43" s="127" t="inlineStr">
+        <is>
+          <t>Found by looking at every screen rather than by a failing test. (1) Every timestamp rendered hours late — the API returns naive UTC and JS reads a suffix-less string as local, so a 3:16 PM capture showed as 8:16 PM; three pages had their own patch, four had none, now one parseUTC. (2) The usage chart plotted only days with calls, so one busy afternoon drew as a solid month-wide bar; now zero-filled. (3) The document graph is a forest of per-feature chains, and top-down put all 24 roots in rank 0 — an unreadable smear; now LR, and it fits on first render. (4) The mind map's 14 controls were one wrapping pile whose dividers separated nothing; now two rows.</t>
+        </is>
+      </c>
+      <c r="E43" s="127" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F43" s="142" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G43" s="142" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H43" s="142" t="inlineStr">
         <is>
           <t>Done</t>
         </is>

</xml_diff>

<commit_message>
docs(roadmap): record the design-system consolidation
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Dobby_100_Day_Roadmap.xlsx
+++ b/Dobby_100_Day_Roadmap.xlsx
@@ -14201,7 +14201,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -15898,6 +15898,46 @@
         </is>
       </c>
       <c r="H43" s="142" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="126" t="n">
+        <v>44</v>
+      </c>
+      <c r="B44" s="142" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="C44" s="142" t="inlineStr">
+        <is>
+          <t>Design system consolidated — one CardHeader, one type scale, one eyebrow</t>
+        </is>
+      </c>
+      <c r="D44" s="127" t="inlineStr">
+        <is>
+          <t>The reskin was applied but not systematised. The titled strip at the top of a card existed 20 times by hand in 8 padding/size combinations; the small-caps label was re-typed at 19 sites in 2 sizes and 2 letter-spacings; and there were 24 distinct type sizes, 10 of them inside a 5px range (10.5, 11.5, 12.5, 13.5, 14.5) — invisible to the eye but not to the browser, so text meant to share a baseline sat on two. Now one CardHeader primitive, .eyebrow everywhere, and 11 sizes with the scale documented in index.css. Two of the 20 headers deliberately kept their own markup: they stack vertically and CardHeader is a horizontal strip.</t>
+        </is>
+      </c>
+      <c r="E44" s="127" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F44" s="142" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G44" s="142" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H44" s="142" t="inlineStr">
         <is>
           <t>Done</t>
         </is>

</xml_diff>